<commit_message>
add new data to combine script
</commit_message>
<xml_diff>
--- a/models.xlsx
+++ b/models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acaug\Documents\School\PhD\lifestage_movement_conservation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7E1993A-B2A3-4F66-92D1-09677E74F296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6285640-D44F-4D3B-9417-CA4AC92067F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1604" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1605" uniqueCount="34">
   <si>
     <t>4 MPA sizes</t>
   </si>
@@ -132,10 +132,13 @@
     <t>MPA Spacing</t>
   </si>
   <si>
-    <t>Done?</t>
+    <t>done</t>
   </si>
   <si>
-    <t>done</t>
+    <t>Simulation</t>
+  </si>
+  <si>
+    <t>Connectivity</t>
   </si>
 </sst>
 </file>
@@ -600,16 +603,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9241C9B2-A5D9-481C-B018-5A593354EEE4}">
-  <dimension ref="A1:L1459"/>
+  <dimension ref="A1:M1459"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.26953125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -638,10 +643,13 @@
         <v>30</v>
       </c>
       <c r="L1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+      <c r="M1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>23</v>
       </c>
@@ -670,10 +678,10 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -702,10 +710,10 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -734,10 +742,10 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -766,10 +774,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -798,10 +806,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -830,10 +838,10 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -862,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -894,10 +902,10 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -926,10 +934,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>23</v>
       </c>
@@ -958,10 +966,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -990,10 +998,10 @@
         <v>0</v>
       </c>
       <c r="L12" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -1022,10 +1030,10 @@
         <v>0</v>
       </c>
       <c r="L13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -1054,10 +1062,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -1086,10 +1094,10 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -1118,7 +1126,7 @@
         <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.35">
@@ -1150,7 +1158,7 @@
         <v>0</v>
       </c>
       <c r="L17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
@@ -1182,7 +1190,7 @@
         <v>0</v>
       </c>
       <c r="L18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
@@ -1214,7 +1222,7 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
@@ -1246,7 +1254,7 @@
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
@@ -1278,7 +1286,7 @@
         <v>0</v>
       </c>
       <c r="L21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
@@ -1310,7 +1318,7 @@
         <v>0</v>
       </c>
       <c r="L22" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
@@ -1342,7 +1350,7 @@
         <v>0</v>
       </c>
       <c r="L23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
@@ -1374,7 +1382,7 @@
         <v>0</v>
       </c>
       <c r="L24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
@@ -1406,7 +1414,7 @@
         <v>0</v>
       </c>
       <c r="L25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.35">
@@ -1438,7 +1446,7 @@
         <v>0</v>
       </c>
       <c r="L26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
@@ -1470,7 +1478,7 @@
         <v>0</v>
       </c>
       <c r="L27" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.35">
@@ -1502,7 +1510,7 @@
         <v>0</v>
       </c>
       <c r="L28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
@@ -1534,7 +1542,7 @@
         <v>0</v>
       </c>
       <c r="L29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.35">
@@ -1566,7 +1574,7 @@
         <v>0</v>
       </c>
       <c r="L30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.35">
@@ -1598,7 +1606,7 @@
         <v>0</v>
       </c>
       <c r="L31" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.35">
@@ -1630,7 +1638,7 @@
         <v>0</v>
       </c>
       <c r="L32" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.35">
@@ -1662,7 +1670,7 @@
         <v>0</v>
       </c>
       <c r="L33" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.35">
@@ -1694,7 +1702,7 @@
         <v>0</v>
       </c>
       <c r="L34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.35">
@@ -1726,7 +1734,7 @@
         <v>0</v>
       </c>
       <c r="L35" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.35">
@@ -1758,7 +1766,7 @@
         <v>0</v>
       </c>
       <c r="L36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.35">
@@ -1790,7 +1798,7 @@
         <v>0</v>
       </c>
       <c r="L37" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.35">
@@ -1822,7 +1830,7 @@
         <v>2</v>
       </c>
       <c r="L38" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.35">
@@ -1854,7 +1862,7 @@
         <v>2</v>
       </c>
       <c r="L39" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.35">
@@ -1886,7 +1894,7 @@
         <v>2</v>
       </c>
       <c r="L40" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.35">
@@ -1918,7 +1926,7 @@
         <v>2</v>
       </c>
       <c r="L41" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.35">
@@ -1950,7 +1958,7 @@
         <v>2</v>
       </c>
       <c r="L42" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.35">
@@ -1982,7 +1990,7 @@
         <v>2</v>
       </c>
       <c r="L43" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.35">
@@ -2014,7 +2022,7 @@
         <v>2</v>
       </c>
       <c r="L44" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.35">
@@ -2046,7 +2054,7 @@
         <v>2</v>
       </c>
       <c r="L45" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.35">
@@ -2078,7 +2086,7 @@
         <v>2</v>
       </c>
       <c r="L46" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.35">
@@ -2110,7 +2118,7 @@
         <v>2</v>
       </c>
       <c r="L47" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.35">
@@ -2142,7 +2150,7 @@
         <v>2</v>
       </c>
       <c r="L48" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.35">
@@ -2174,7 +2182,7 @@
         <v>2</v>
       </c>
       <c r="L49" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.35">
@@ -2206,7 +2214,7 @@
         <v>2</v>
       </c>
       <c r="L50" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.35">
@@ -2238,7 +2246,7 @@
         <v>2</v>
       </c>
       <c r="L51" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.35">
@@ -2270,7 +2278,7 @@
         <v>2</v>
       </c>
       <c r="L52" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.35">
@@ -2302,7 +2310,7 @@
         <v>2</v>
       </c>
       <c r="L53" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.35">
@@ -2334,7 +2342,7 @@
         <v>2</v>
       </c>
       <c r="L54" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.35">
@@ -2366,7 +2374,7 @@
         <v>2</v>
       </c>
       <c r="L55" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.35">
@@ -2398,7 +2406,7 @@
         <v>4</v>
       </c>
       <c r="L56" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.35">
@@ -2430,7 +2438,7 @@
         <v>4</v>
       </c>
       <c r="L57" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.35">
@@ -2462,7 +2470,7 @@
         <v>4</v>
       </c>
       <c r="L58" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.35">
@@ -2494,7 +2502,7 @@
         <v>4</v>
       </c>
       <c r="L59" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.35">
@@ -2526,7 +2534,7 @@
         <v>4</v>
       </c>
       <c r="L60" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.35">
@@ -2558,7 +2566,7 @@
         <v>4</v>
       </c>
       <c r="L61" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.35">
@@ -2590,7 +2598,7 @@
         <v>4</v>
       </c>
       <c r="L62" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.35">
@@ -2622,7 +2630,7 @@
         <v>4</v>
       </c>
       <c r="L63" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.35">
@@ -2654,7 +2662,7 @@
         <v>4</v>
       </c>
       <c r="L64" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.35">
@@ -2686,7 +2694,7 @@
         <v>4</v>
       </c>
       <c r="L65" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.35">
@@ -2718,7 +2726,7 @@
         <v>4</v>
       </c>
       <c r="L66" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.35">
@@ -2750,7 +2758,7 @@
         <v>4</v>
       </c>
       <c r="L67" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.35">
@@ -2782,7 +2790,7 @@
         <v>4</v>
       </c>
       <c r="L68" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.35">
@@ -2814,7 +2822,7 @@
         <v>4</v>
       </c>
       <c r="L69" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.35">
@@ -2846,7 +2854,7 @@
         <v>4</v>
       </c>
       <c r="L70" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.35">
@@ -2878,7 +2886,7 @@
         <v>4</v>
       </c>
       <c r="L71" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.35">
@@ -2910,7 +2918,7 @@
         <v>4</v>
       </c>
       <c r="L72" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.35">
@@ -2942,7 +2950,7 @@
         <v>4</v>
       </c>
       <c r="L73" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.35">
@@ -2974,7 +2982,7 @@
         <v>8</v>
       </c>
       <c r="L74" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.35">
@@ -3006,7 +3014,7 @@
         <v>8</v>
       </c>
       <c r="L75" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.35">
@@ -3038,7 +3046,7 @@
         <v>8</v>
       </c>
       <c r="L76" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.35">
@@ -3070,7 +3078,7 @@
         <v>8</v>
       </c>
       <c r="L77" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.35">
@@ -3102,7 +3110,7 @@
         <v>8</v>
       </c>
       <c r="L78" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.35">
@@ -3134,7 +3142,7 @@
         <v>8</v>
       </c>
       <c r="L79" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.35">
@@ -3166,7 +3174,7 @@
         <v>8</v>
       </c>
       <c r="L80" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.35">
@@ -3198,7 +3206,7 @@
         <v>8</v>
       </c>
       <c r="L81" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.35">
@@ -3230,7 +3238,7 @@
         <v>8</v>
       </c>
       <c r="L82" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.35">
@@ -3262,7 +3270,7 @@
         <v>8</v>
       </c>
       <c r="L83" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.35">
@@ -3294,7 +3302,7 @@
         <v>8</v>
       </c>
       <c r="L84" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.35">
@@ -3326,7 +3334,7 @@
         <v>8</v>
       </c>
       <c r="L85" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.35">
@@ -3358,7 +3366,7 @@
         <v>8</v>
       </c>
       <c r="L86" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.35">
@@ -3390,7 +3398,7 @@
         <v>8</v>
       </c>
       <c r="L87" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.35">
@@ -3422,7 +3430,7 @@
         <v>8</v>
       </c>
       <c r="L88" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.35">
@@ -3454,7 +3462,7 @@
         <v>8</v>
       </c>
       <c r="L89" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.35">
@@ -3486,7 +3494,7 @@
         <v>8</v>
       </c>
       <c r="L90" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.35">
@@ -3518,7 +3526,7 @@
         <v>8</v>
       </c>
       <c r="L91" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.35">
@@ -3550,7 +3558,7 @@
         <v>16</v>
       </c>
       <c r="L92" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.35">
@@ -3582,7 +3590,7 @@
         <v>16</v>
       </c>
       <c r="L93" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.35">
@@ -3614,7 +3622,7 @@
         <v>16</v>
       </c>
       <c r="L94" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95" spans="1:12" x14ac:dyDescent="0.35">
@@ -3646,7 +3654,7 @@
         <v>16</v>
       </c>
       <c r="L95" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.35">
@@ -3678,7 +3686,7 @@
         <v>16</v>
       </c>
       <c r="L96" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.35">
@@ -3710,7 +3718,7 @@
         <v>16</v>
       </c>
       <c r="L97" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.35">
@@ -3742,7 +3750,7 @@
         <v>16</v>
       </c>
       <c r="L98" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="99" spans="1:12" x14ac:dyDescent="0.35">
@@ -3774,7 +3782,7 @@
         <v>16</v>
       </c>
       <c r="L99" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.35">
@@ -3806,7 +3814,7 @@
         <v>16</v>
       </c>
       <c r="L100" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="101" spans="1:12" x14ac:dyDescent="0.35">
@@ -3838,7 +3846,7 @@
         <v>16</v>
       </c>
       <c r="L101" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.35">
@@ -3870,7 +3878,7 @@
         <v>16</v>
       </c>
       <c r="L102" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="103" spans="1:12" x14ac:dyDescent="0.35">
@@ -3902,7 +3910,7 @@
         <v>16</v>
       </c>
       <c r="L103" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="104" spans="1:12" x14ac:dyDescent="0.35">
@@ -3934,7 +3942,7 @@
         <v>16</v>
       </c>
       <c r="L104" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.35">
@@ -3966,7 +3974,7 @@
         <v>16</v>
       </c>
       <c r="L105" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.35">
@@ -3998,7 +4006,7 @@
         <v>16</v>
       </c>
       <c r="L106" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.35">
@@ -4030,7 +4038,7 @@
         <v>16</v>
       </c>
       <c r="L107" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.35">
@@ -4062,7 +4070,7 @@
         <v>16</v>
       </c>
       <c r="L108" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.35">
@@ -4094,7 +4102,7 @@
         <v>16</v>
       </c>
       <c r="L109" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
get all models run
</commit_message>
<xml_diff>
--- a/models.xlsx
+++ b/models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acaug\Documents\School\PhD\lifestage_movement_conservation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6285640-D44F-4D3B-9417-CA4AC92067F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5374E290-13CC-4EC8-B646-C6F306D80AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1605" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1713" uniqueCount="34">
   <si>
     <t>4 MPA sizes</t>
   </si>
@@ -680,6 +680,9 @@
       <c r="L2" t="s">
         <v>31</v>
       </c>
+      <c r="M2" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -712,6 +715,9 @@
       <c r="L3" t="s">
         <v>31</v>
       </c>
+      <c r="M3" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -744,6 +750,9 @@
       <c r="L4" t="s">
         <v>31</v>
       </c>
+      <c r="M4" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -776,6 +785,9 @@
       <c r="L5" t="s">
         <v>31</v>
       </c>
+      <c r="M5" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -808,6 +820,9 @@
       <c r="L6" t="s">
         <v>31</v>
       </c>
+      <c r="M6" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -838,6 +853,9 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
+        <v>31</v>
+      </c>
+      <c r="M7" t="s">
         <v>31</v>
       </c>
     </row>
@@ -872,6 +890,9 @@
       <c r="L8" t="s">
         <v>31</v>
       </c>
+      <c r="M8" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -904,6 +925,9 @@
       <c r="L9" t="s">
         <v>31</v>
       </c>
+      <c r="M9" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
@@ -936,6 +960,9 @@
       <c r="L10" t="s">
         <v>31</v>
       </c>
+      <c r="M10" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
@@ -968,6 +995,9 @@
       <c r="L11" t="s">
         <v>31</v>
       </c>
+      <c r="M11" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -1000,6 +1030,9 @@
       <c r="L12" t="s">
         <v>31</v>
       </c>
+      <c r="M12" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
@@ -1032,6 +1065,9 @@
       <c r="L13" t="s">
         <v>31</v>
       </c>
+      <c r="M13" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
@@ -1064,6 +1100,9 @@
       <c r="L14" t="s">
         <v>31</v>
       </c>
+      <c r="M14" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
@@ -1096,6 +1135,9 @@
       <c r="L15" t="s">
         <v>31</v>
       </c>
+      <c r="M15" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -1128,8 +1170,11 @@
       <c r="L16" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>28</v>
       </c>
@@ -1160,8 +1205,11 @@
       <c r="L17" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -1192,8 +1240,11 @@
       <c r="L18" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>27</v>
       </c>
@@ -1224,8 +1275,11 @@
       <c r="L19" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M19" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>23</v>
       </c>
@@ -1256,8 +1310,11 @@
       <c r="L20" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>15</v>
       </c>
@@ -1288,8 +1345,11 @@
       <c r="L21" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M21" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>24</v>
       </c>
@@ -1320,8 +1380,11 @@
       <c r="L22" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>25</v>
       </c>
@@ -1352,8 +1415,11 @@
       <c r="L23" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M23" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>26</v>
       </c>
@@ -1384,8 +1450,11 @@
       <c r="L24" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M24" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>16</v>
       </c>
@@ -1416,8 +1485,11 @@
       <c r="L25" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -1448,8 +1520,11 @@
       <c r="L26" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M26" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>17</v>
       </c>
@@ -1480,8 +1555,11 @@
       <c r="L27" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M27" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -1512,8 +1590,11 @@
       <c r="L28" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M28" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>23</v>
       </c>
@@ -1544,8 +1625,11 @@
       <c r="L29" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M29" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>15</v>
       </c>
@@ -1576,8 +1660,11 @@
       <c r="L30" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M30" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>24</v>
       </c>
@@ -1608,8 +1695,11 @@
       <c r="L31" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M31" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>25</v>
       </c>
@@ -1640,8 +1730,11 @@
       <c r="L32" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>26</v>
       </c>
@@ -1672,8 +1765,11 @@
       <c r="L33" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M33" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>16</v>
       </c>
@@ -1704,8 +1800,11 @@
       <c r="L34" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M34" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>28</v>
       </c>
@@ -1736,8 +1835,11 @@
       <c r="L35" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M35" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>17</v>
       </c>
@@ -1768,8 +1870,11 @@
       <c r="L36" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M36" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>27</v>
       </c>
@@ -1800,8 +1905,11 @@
       <c r="L37" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M37" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>23</v>
       </c>
@@ -1832,8 +1940,11 @@
       <c r="L38" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M38" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>15</v>
       </c>
@@ -1864,8 +1975,11 @@
       <c r="L39" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M39" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>24</v>
       </c>
@@ -1896,8 +2010,11 @@
       <c r="L40" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M40" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>25</v>
       </c>
@@ -1928,8 +2045,11 @@
       <c r="L41" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M41" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>26</v>
       </c>
@@ -1960,8 +2080,11 @@
       <c r="L42" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M42" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>16</v>
       </c>
@@ -1992,8 +2115,11 @@
       <c r="L43" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M43" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>28</v>
       </c>
@@ -2024,8 +2150,11 @@
       <c r="L44" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M44" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>17</v>
       </c>
@@ -2056,8 +2185,11 @@
       <c r="L45" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M45" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>27</v>
       </c>
@@ -2088,8 +2220,11 @@
       <c r="L46" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M46" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>23</v>
       </c>
@@ -2120,8 +2255,11 @@
       <c r="L47" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M47" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>15</v>
       </c>
@@ -2152,8 +2290,11 @@
       <c r="L48" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M48" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>24</v>
       </c>
@@ -2184,8 +2325,11 @@
       <c r="L49" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M49" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>25</v>
       </c>
@@ -2216,8 +2360,11 @@
       <c r="L50" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M50" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>26</v>
       </c>
@@ -2248,8 +2395,11 @@
       <c r="L51" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M51" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>16</v>
       </c>
@@ -2280,8 +2430,11 @@
       <c r="L52" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M52" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>28</v>
       </c>
@@ -2312,8 +2465,11 @@
       <c r="L53" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M53" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>17</v>
       </c>
@@ -2344,8 +2500,11 @@
       <c r="L54" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M54" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>27</v>
       </c>
@@ -2376,8 +2535,11 @@
       <c r="L55" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M55" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>23</v>
       </c>
@@ -2408,8 +2570,11 @@
       <c r="L56" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M56" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>15</v>
       </c>
@@ -2440,8 +2605,11 @@
       <c r="L57" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M57" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>24</v>
       </c>
@@ -2472,8 +2640,11 @@
       <c r="L58" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M58" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>25</v>
       </c>
@@ -2504,8 +2675,11 @@
       <c r="L59" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M59" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>26</v>
       </c>
@@ -2536,8 +2710,11 @@
       <c r="L60" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M60" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>16</v>
       </c>
@@ -2568,8 +2745,11 @@
       <c r="L61" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M61" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>28</v>
       </c>
@@ -2600,8 +2780,11 @@
       <c r="L62" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M62" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>17</v>
       </c>
@@ -2632,8 +2815,11 @@
       <c r="L63" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M63" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>27</v>
       </c>
@@ -2664,8 +2850,11 @@
       <c r="L64" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M64" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>23</v>
       </c>
@@ -2696,8 +2885,11 @@
       <c r="L65" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M65" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>15</v>
       </c>
@@ -2728,8 +2920,11 @@
       <c r="L66" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M66" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>24</v>
       </c>
@@ -2760,8 +2955,11 @@
       <c r="L67" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M67" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>25</v>
       </c>
@@ -2792,8 +2990,11 @@
       <c r="L68" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M68" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>26</v>
       </c>
@@ -2824,8 +3025,11 @@
       <c r="L69" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M69" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>16</v>
       </c>
@@ -2856,8 +3060,11 @@
       <c r="L70" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M70" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>28</v>
       </c>
@@ -2888,8 +3095,11 @@
       <c r="L71" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M71" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>17</v>
       </c>
@@ -2920,8 +3130,11 @@
       <c r="L72" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M72" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>27</v>
       </c>
@@ -2952,8 +3165,11 @@
       <c r="L73" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M73" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>23</v>
       </c>
@@ -2984,8 +3200,11 @@
       <c r="L74" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M74" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>15</v>
       </c>
@@ -3016,8 +3235,11 @@
       <c r="L75" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M75" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>24</v>
       </c>
@@ -3048,8 +3270,11 @@
       <c r="L76" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M76" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>25</v>
       </c>
@@ -3080,8 +3305,11 @@
       <c r="L77" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M77" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>26</v>
       </c>
@@ -3112,8 +3340,11 @@
       <c r="L78" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M78" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>16</v>
       </c>
@@ -3144,8 +3375,11 @@
       <c r="L79" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M79" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>28</v>
       </c>
@@ -3176,8 +3410,11 @@
       <c r="L80" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M80" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>17</v>
       </c>
@@ -3208,8 +3445,11 @@
       <c r="L81" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M81" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="82" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>27</v>
       </c>
@@ -3240,8 +3480,11 @@
       <c r="L82" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M82" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="83" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>23</v>
       </c>
@@ -3272,8 +3515,11 @@
       <c r="L83" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M83" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="84" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>15</v>
       </c>
@@ -3304,8 +3550,11 @@
       <c r="L84" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M84" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="85" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>24</v>
       </c>
@@ -3336,8 +3585,11 @@
       <c r="L85" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M85" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>25</v>
       </c>
@@ -3368,8 +3620,11 @@
       <c r="L86" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M86" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="87" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>26</v>
       </c>
@@ -3400,8 +3655,11 @@
       <c r="L87" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M87" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="88" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>16</v>
       </c>
@@ -3432,8 +3690,11 @@
       <c r="L88" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M88" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="89" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>28</v>
       </c>
@@ -3464,8 +3725,11 @@
       <c r="L89" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M89" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="90" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>17</v>
       </c>
@@ -3496,8 +3760,11 @@
       <c r="L90" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M90" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="91" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>27</v>
       </c>
@@ -3528,8 +3795,11 @@
       <c r="L91" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M91" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="92" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>23</v>
       </c>
@@ -3560,8 +3830,11 @@
       <c r="L92" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M92" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="93" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>15</v>
       </c>
@@ -3592,8 +3865,11 @@
       <c r="L93" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M93" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="94" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>24</v>
       </c>
@@ -3624,8 +3900,11 @@
       <c r="L94" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M94" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="95" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>25</v>
       </c>
@@ -3656,8 +3935,11 @@
       <c r="L95" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M95" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="96" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>26</v>
       </c>
@@ -3688,8 +3970,11 @@
       <c r="L96" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M96" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="97" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>16</v>
       </c>
@@ -3720,8 +4005,11 @@
       <c r="L97" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M97" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="98" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>28</v>
       </c>
@@ -3752,8 +4040,11 @@
       <c r="L98" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M98" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="99" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>17</v>
       </c>
@@ -3784,8 +4075,11 @@
       <c r="L99" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M99" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="100" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>27</v>
       </c>
@@ -3816,8 +4110,11 @@
       <c r="L100" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M100" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="101" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>23</v>
       </c>
@@ -3848,8 +4145,11 @@
       <c r="L101" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M101" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="102" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>15</v>
       </c>
@@ -3880,8 +4180,11 @@
       <c r="L102" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M102" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="103" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>24</v>
       </c>
@@ -3912,8 +4215,11 @@
       <c r="L103" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M103" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="104" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>25</v>
       </c>
@@ -3944,8 +4250,11 @@
       <c r="L104" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M104" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="105" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>26</v>
       </c>
@@ -3976,8 +4285,11 @@
       <c r="L105" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M105" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="106" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>16</v>
       </c>
@@ -4008,8 +4320,11 @@
       <c r="L106" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M106" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="107" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>28</v>
       </c>
@@ -4040,8 +4355,11 @@
       <c r="L107" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M107" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="108" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>17</v>
       </c>
@@ -4072,8 +4390,11 @@
       <c r="L108" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M108" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="109" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>27</v>
       </c>
@@ -4104,8 +4425,11 @@
       <c r="L109" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M109" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="110" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>23</v>
       </c>
@@ -4122,7 +4446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>15</v>
       </c>
@@ -4139,7 +4463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>24</v>
       </c>

</xml_diff>

<commit_message>
change inside out side name
</commit_message>
<xml_diff>
--- a/models.xlsx
+++ b/models.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acaug\Documents\School\PhD\lifestage_movement_conservation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C3230C0-E220-4E41-856C-5F8C81B9D920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B01AD6D4-6A39-4DBD-887D-099D0F07E343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1052,6 +1052,10 @@
       <c r="E15">
         <v>0</v>
       </c>
+      <c r="J15">
+        <f>3 *3 *3 * 3 * 4 * 5</f>
+        <v>1620</v>
+      </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" t="s">

</xml_diff>